<commit_message>
fix(schedules): giờ có mặt tại kho bắt buộc, giờ xuất phát không còn mất trắng khi thiếu phút bốc hàng
- _compute_planned_departure (api/schedules.py + bản sao seed_demo_data.py) chỉ
  còn cần depot_arrival_time để tính giờ xuất phát; thiếu depot_loading_duration_min
  coi như bốc 0 phút thay vì trả None.
- depot_arrival_time chuyển bắt buộc ở cả form nhập tay (Pydantic 422) và Excel
  upload (chặn cả file, báo đúng hàng thiếu) — trước đây thiếu chỉ âm thầm làm
  Dashboard mất dòng "xuất phát HH:MM" không ai biết.
- Cập nhật schedule_template.xlsx + TECHNICAL_SPEC.md theo đúng luật mới.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/schedule_template.xlsx
+++ b/schedule_template.xlsx
@@ -874,12 +874,13 @@
       <c r="D2" s="15" t="inlineStr">
         <is>
           <t>Giờ có mặt tại kho
-(HH:MM) **</t>
+(HH:MM) ** — BẮT BUỘC</t>
         </is>
       </c>
       <c r="E2" s="15" t="inlineStr">
         <is>
-          <t>Phút bốc hàng tại kho **</t>
+          <t>Phút bốc hàng tại kho **
+— để trống = 0 phút</t>
         </is>
       </c>
       <c r="F2" s="12" t="inlineStr">
@@ -1303,7 +1304,7 @@
       </c>
       <c r="B8" s="18" t="inlineStr">
         <is>
-          <t>depot_arrival_time và depot_loading_duration_min CHỈ điền ở hàng đầu tiên của chuyến (không forward-fill như 3 cột trên — 2 cột này chỉ có ý nghĩa ở đúng 1 thời điểm đầu chuyến). Hệ thống tự tính giờ xuất phát = depot_arrival_time + depot_loading_duration_min, KHÔNG có cột riêng để nhập giờ xuất phát.</t>
+          <t>depot_arrival_time và depot_loading_duration_min CHỈ điền ở hàng đầu tiên của chuyến (không forward-fill như 3 cột trên — 2 cột này chỉ có ý nghĩa ở đúng 1 thời điểm đầu chuyến). depot_arrival_time là BẮT BUỘC ở hàng đầu tiên của mỗi chuyến: thiếu nó thì không tính được giờ xuất phát, upload sẽ bị chặn kèm số hàng cụ thể. depot_loading_duration_min không bắt buộc — để trống = bốc hàng 0 phút, tức xuất phát ngay khi có mặt tại kho. Hệ thống tự tính giờ xuất phát = depot_arrival_time + depot_loading_duration_min, KHÔNG có cột riêng để nhập giờ xuất phát.</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1352,7 @@
       </c>
       <c r="B12" s="18" t="inlineStr">
         <is>
-          <t>Xanh dương đậm = bắt buộc. Xanh lá = không bắt buộc. Vàng cam = chỉ bắt buộc/có ý nghĩa ở hàng đầu tiên của chuyến (Ke_hoach_giao_hang).</t>
+          <t>Xanh dương đậm = bắt buộc. Xanh lá = không bắt buộc. Vàng cam = chỉ điền ở hàng đầu tiên của chuyến (Ke_hoach_giao_hang) — trong đó depot_arrival_time là bắt buộc, depot_loading_duration_min thì không.</t>
         </is>
       </c>
     </row>

</xml_diff>